<commit_message>
263-case catalog; media/one-sided/flawed charts; scrutiny, referrals, impeachments; Biden bank reports + foreign money; NY fraud + Mar-a-Lago charts; essay trims; beta banner; new opening statement
</commit_message>
<xml_diff>
--- a/backup-2026-09-26/site-from-checkpoint/public_html/downloads/first-term-trump-admin-media-deception.xlsx
+++ b/backup-2026-09-26/site-from-checkpoint/public_html/downloads/first-term-trump-admin-media-deception.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="First Term 2017-2021" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="First Term 2017-2021" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'First Term 2017-2021'!$A$1:$L$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'First Term 2017-2021'!$A$1:$L$149</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L143"/>
+  <dimension ref="A1:L149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -9173,8 +9173,386 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Posted a crime graphic claiming “Whites killed by blacks — 81%” and “Whites killed by whites — 16%.”
+Began: Nov 22, 2015 | Ended: never corrected</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>https://www.politifact.com/article/2015/dec/21/2015-lie-year-donald-trump-campaign-misstatements/</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Donald Trump (2016 campaign), Twitter post</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>repeated / never corrected</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>fabricated statistic</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>254</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>Primary record: FBI Expanded Homicide Data Table 6 (2014), white victims: 3,021 total; 2,488 white offenders (82.4%); 446 Black offenders (14.8%). The graphic's 81% and 16% are wrong.</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>Proven false</t>
+        </is>
+      </c>
+      <c r="J144" s="3" t="inlineStr">
+        <is>
+          <t>https://ucr.fbi.gov/crime-in-the-u.s/2014/crime-in-the-u.s.-2014/tables/expanded-homicide-data/expanded_homicide_data_table_6_murder_race_and_sex_of_vicitm_by_race_and_sex_of_offender_2014.xls</t>
+        </is>
+      </c>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>Official record</t>
+        </is>
+      </c>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>Never corrected — fact-checked only</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Said the U.S. has a “$500 billion a year trade deficit with China.”
+Began: Mar 7, 2016 | Ended: repeated</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>https://www.politico.com/magazine/story/2016/03/trump-fact-check-errors-exaggerations-falsehoods-213730</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Donald Trump (2016 campaign), rally in Concord, N.C.</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>repeated / never corrected</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>inflated number</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>Primary record: Census: “The deficit with China increased $22.6 billion to $365.7 billion in 2015.” BEA gives the same $365.7 billion.</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>Proven false</t>
+        </is>
+      </c>
+      <c r="J145" s="3" t="inlineStr">
+        <is>
+          <t>https://www.census.gov/newsroom/blogs/global-reach/2016/02/the-goods-and-services-deficit-increased-to-43-4-billion-in-december-2015.html</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>Official record</t>
+        </is>
+      </c>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>Never corrected — fact-checked only</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Said: “I did not email any classified material to anyone on my email. There is no classified material.”
+Began: Mar 10, 2015 | Ended: never corrected</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>https://www.factcheck.org/2016/08/clintons-email-falsehood/</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Hillary Clinton (D), news conference</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>repeated / never corrected</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>false denial</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>Primary record: FBI Director Comey, July 5, 2016: 110 emails in 52 email chains contained classified information at the time they were sent or received.</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>Proven false</t>
+        </is>
+      </c>
+      <c r="J146" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fbi.gov/news/press-releases/fbi-releases-documents-in-hillary-clinton-e-mail-investigation</t>
+        </is>
+      </c>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>Official record</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>Never corrected — fact-checked only</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>Said: “Director Comey said my answers were truthful.”
+Began: Jul 31, 2016 | Ended: never corrected</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>https://www.factcheck.org/2016/08/clintons-email-falsehood/</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Hillary Clinton (D), Fox News Sunday interview</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>repeated / never corrected</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>misquote / mischaracterization</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>257</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>Primary record: Comey said only that there was no basis to conclude she lied to the FBI; asked about her public statements he said “There was classified material emailed.”</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>Proven false</t>
+        </is>
+      </c>
+      <c r="J147" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fbi.gov/news/press-releases/fbi-releases-documents-in-hillary-clinton-e-mail-investigation</t>
+        </is>
+      </c>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>Official record</t>
+        </is>
+      </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>Never corrected — fact-checked only</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Said the inauguration drew “the largest audience to ever witness an inauguration — period — both in person and around the globe.”
+Began: Jan 21, 2017 | Ended: never corrected</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>https://www.factcheck.org/2017/01/the-facts-on-crowd-size/</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Sean Spicer, White House press secretary (R)</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>repeated / never corrected</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>exaggeration</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>misleading</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>258</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>Primary record: WMATA Metro ridership: 570,557 full-day trips in 2017 vs 782,000 (2013) and 1.1 million (2009). The in-person claim is contradicted; no official global audience count exists.</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>Rated misleading</t>
+        </is>
+      </c>
+      <c r="J148" s="3" t="inlineStr">
+        <is>
+          <t>https://trumpwhitehouse.archives.gov/briefings-statements/statement-press-secretary-sean-spicer/</t>
+        </is>
+      </c>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>Official record</t>
+        </is>
+      </c>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>Never corrected — fact-checked only</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>Claimed the CDC “quietly updated the Covid number to admit that only 6% of all the 153,504 deaths recorded actually died from Covid.”
+Began: Aug 30, 2020 | Ended: post removed by Twitter</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>https://www.factcheck.org/2020/09/cdc-did-not-admit-only-6-of-recorded-deaths-from-covid-19/</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Viral social media post (shared by Donald Trump on Twitter)</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>repeated / never corrected</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>misread statistic</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>259</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>Primary record: CDC: over 5% of COVID-19 death certificates listed COVID-19 as the only cause; the rest averaged 4.0 additional conditions. The 6% never meant only 6% died from COVID-19.</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>Proven false</t>
+        </is>
+      </c>
+      <c r="J149" s="3" t="inlineStr">
+        <is>
+          <t>https://www.factcheck.org/2020/09/cdc-did-not-admit-only-6-of-recorded-deaths-from-covid-19/</t>
+        </is>
+      </c>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>Official record</t>
+        </is>
+      </c>
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>Never corrected — fact-checked only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L143"/>
+  <autoFilter ref="A1:L149"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
@@ -9471,6 +9849,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B143" r:id="rId293"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="rId294"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J143" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J144" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J145" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B146" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J146" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B147" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J147" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B148" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J148" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J149" r:id="rId307"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>